<commit_message>
Sprint 13 finished: Railway/Vercel Deployment ready
</commit_message>
<xml_diff>
--- a/documentacion/Plan de pruebas examen/plan-de-pruebas.xlsx
+++ b/documentacion/Plan de pruebas examen/plan-de-pruebas.xlsx
@@ -506,14 +506,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alcance: pruebas automatizadas de backend e IA (Sprint 12) y pruebas manuales E2E del flujo core (Sprint 13). Estado del plan: 22/22 casos ejecutados.</t>
+          <t>Alcance: pruebas automatizadas de backend e IA (Sprint 12) y validación manual del despliegue cloud y demo del flujo core (Sprint 13). Estado del plan: 22/22 casos ejecutados.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Entorno de pruebas: local con Java 21, Maven, Python 3.11, Docker Desktop. Integración backend usa Testcontainers (MySQL + imagen ai-service) o WORKSI_IT_AI_URL apuntando a IA en localhost:8000.</t>
+          <t>Entorno de pruebas: local con Java 21, Maven, Python 3.11, Docker Desktop (Sprint 12). Integración backend usa Testcontainers (MySQL + imagen ai-service) o WORKSI_IT_AI_URL apuntando a IA en localhost:8000. Sprint 13: entorno cloud Vercel (web) + Railway (MySQL, backend, IA); app móvil con BASE_URL HTTPS del backend.</t>
         </is>
       </c>
     </row>
@@ -527,14 +527,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Criterio de éxito general: cada caso de la tabla cumple su resultado esperado; bugs críticos (caídas, 500 en flujo core, datos cruzados, score inconsistente, mensajes a terceros) deben quedar en cero antes de la demo stakeholder.</t>
+          <t>Criterio de éxito general: cada caso de la tabla cumple su resultado esperado; bugs críticos (caídas, 500 en flujo core en cloud, proxy /api roto, BD no migrada, score inconsistente, mensajes a terceros) deben quedar en cero antes de la demo stakeholder.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Evidencias (TP-01 a TP-22): capturas en la sección 6 de este documento. TP-01 a TP-13: tres capturas de terminal (EV-UNIT, EV-INT, EV-IA). TP-14 a TP-22: capturas E2E del producto.</t>
+          <t>Evidencias (TP-01 a TP-22): capturas en la sección 6 de este documento. TP-01 a TP-13: tres capturas de terminal (EV-UNIT, EV-INT, EV-IA). TP-14 a TP-22: capturas de validación cloud y demo del producto.</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>E2E — Admin</t>
+          <t>Cloud — Admin</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Manual funcional (E2E)</t>
+          <t>Manual funcional (cloud)</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Con Docker Compose: login ADMIN; crear empresa multipart; crear reclutador asociado.</t>
+          <t>En portal web Vercel: login ADMIN; crear empresa multipart; crear reclutador asociado (API vía proxy /api).</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>E2E — Candidato móvil</t>
+          <t>Cloud — Candidato móvil</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1336,12 +1336,12 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Manual funcional (E2E)</t>
+          <t>Manual funcional (cloud)</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>App Android: consentimiento HU-21; registro con CV PDF y datos perfil.</t>
+          <t>App Android con BASE_URL backend Railway: consentimiento HU-21; registro con CV PDF y datos perfil.</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>E2E — Reclutador web</t>
+          <t>Cloud — Reclutador web</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1388,12 +1388,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Manual funcional (E2E)</t>
+          <t>Manual funcional (cloud)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Portal RECRUITER: crear oferta con campos obligatorios y skills.</t>
+          <t>Portal RECRUITER en Vercel: crear oferta con campos obligatorios y skills.</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>E2E — Candidato móvil</t>
+          <t>Cloud — Candidato móvil</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1440,12 +1440,12 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Manual funcional (E2E)</t>
+          <t>Manual funcional (cloud)</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Candidato autenticado: feed con score; swipe APPLY; confirmar postulación.</t>
+          <t>Candidato autenticado contra API Railway: feed con score; swipe APPLY; confirmar postulación.</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>E2E — Reclutador web</t>
+          <t>Cloud — Reclutador web</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1492,12 +1492,12 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Manual funcional (E2E)</t>
+          <t>Manual funcional (cloud)</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Reclutador: listado postulantes; abrir detalle; ver cinco dimensiones y score.</t>
+          <t>Reclutador en Vercel: listado postulantes; abrir detalle; ver cinco dimensiones y score.</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>E2E — Match y mensajería</t>
+          <t>Cloud — Match y mensajería</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1544,12 +1544,12 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Manual funcional (E2E)</t>
+          <t>Manual funcional (cloud)</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Reclutador: Establecer Match con primer mensaje; bandeja Matchs; hilo mensajes. Candidato: aviso post-login; Matchs; responder.</t>
+          <t>Reclutador web: Establecer Match con primer mensaje; bandeja Matchs; hilo mensajes. Candidato móvil: aviso post-login; Matchs; responder.</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>E2E — Matching</t>
+          <t>Cloud — Matching</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Misma oferta y mismo CV: cambiar solo skills perfil u oferta; comparar score antes/después (complementa TP-10).</t>
+          <t>En entorno cloud: misma oferta y mismo CV; cambiar solo skills perfil u oferta; comparar score antes/después (complementa TP-10 / Sprint 12).</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Cloud — Infraestructura</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Ambiente reproducible Docker</t>
+          <t>Despliegue Vercel + Railway (Sprint 13)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1653,22 +1653,22 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>En máquina limpia: docker compose up según producto/README.md; verificar mysql, backend, ai-service.</t>
+          <t>Tras deploy: GET /health backend e IA en Railway; portal web Vercel accesible; rewrite /api hacia backend; volumen CV montado en backend.</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>docker-compose.yml del repositorio</t>
+          <t>Servicios Railway (MySQL, backend, ai-service) y proyecto Vercel frontWeb</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Servicios levantan; /health IA responde; backend accesible.</t>
+          <t>Health UP; web carga; API responde vía proxy; backend persiste CV.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>docker compose up con contenedores activos; GET /health IA responde OK. Ver §6.2 (EV-21).</t>
+          <t>Health backend e IA OK; web Vercel operativa; proxy /api funcional. Ver §6.2 (EV-21).</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>§6.2 — EV-21: capturas Docker y /health</t>
+          <t>§6.2 — EV-21: capturas health y portal web</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Cloud — Seguridad</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Sin token: GET rutas protegidas → 401. Con JWT incorrecto rol → 403 donde aplique.</t>
+          <t>Contra URL pública del backend Railway: sin token GET rutas protegidas → 401; con JWT rol incorrecto → 403 donde aplique.</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -1808,7 +1808,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Pruebas manuales E2E y operativas</t>
+          <t>Pruebas manuales cloud y demo (Sprint 13)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>